<commit_message>
Complete Brazil 2011–2024 oil trade balance in saldo workbook
Fill import dispendio from ANP yearbook so Brazil annual balances
cover the full 2011–2026 window alongside Petrobras.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/anp/saldo_petroleo_export_import/saldo_petroleo_export_import_2011_2026.xlsx
+++ b/anp/saldo_petroleo_export_import/saldo_petroleo_export_import_2011_2026.xlsx
@@ -834,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -861,29 +861,225 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2025</v>
+        <v>2011</v>
       </c>
       <c r="B2" t="n">
-        <v>44536157927</v>
+        <v>21785444945</v>
       </c>
       <c r="C2" t="n">
-        <v>6611866628</v>
+        <v>14151806000</v>
       </c>
       <c r="D2" t="n">
-        <v>37924291299</v>
+        <v>7633638945</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B3" t="n">
+        <v>20305876591</v>
+      </c>
+      <c r="C3" t="n">
+        <v>13448477370</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6857399221</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B4" t="n">
+        <v>12956607442</v>
+      </c>
+      <c r="C4" t="n">
+        <v>16463302900</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-3506695458</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B5" t="n">
+        <v>16356739584</v>
+      </c>
+      <c r="C5" t="n">
+        <v>15873935470</v>
+      </c>
+      <c r="D5" t="n">
+        <v>482804114</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B6" t="n">
+        <v>11781308300</v>
+      </c>
+      <c r="C6" t="n">
+        <v>7380844000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4400464300</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B7" t="n">
+        <v>10073797268</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2898855786</v>
+      </c>
+      <c r="D7" t="n">
+        <v>7174941482</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B8" t="n">
+        <v>16624996815</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2966954176</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13658042639</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B9" t="n">
+        <v>25096773303</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5042501227</v>
+      </c>
+      <c r="D9" t="n">
+        <v>20054272076</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B10" t="n">
+        <v>24002331852</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4651641478</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19350690374</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B11" t="n">
+        <v>19613857907</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2613731569</v>
+      </c>
+      <c r="D11" t="n">
+        <v>17000126338</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B12" t="n">
+        <v>30608981653</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3995255654</v>
+      </c>
+      <c r="D12" t="n">
+        <v>26613725999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B13" t="n">
+        <v>42553764089</v>
+      </c>
+      <c r="C13" t="n">
+        <v>9914865806</v>
+      </c>
+      <c r="D13" t="n">
+        <v>32638898283</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B14" t="n">
+        <v>42611078672</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9058456152</v>
+      </c>
+      <c r="D14" t="n">
+        <v>33552622520</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B15" t="n">
+        <v>44963878520</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8690210062</v>
+      </c>
+      <c r="D15" t="n">
+        <v>36273668458</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B16" t="n">
+        <v>44536157927</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6611866628</v>
+      </c>
+      <c r="D16" t="n">
+        <v>37924291299</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
         <v>2026</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B17" t="n">
         <v>27903018706</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C17" t="n">
         <v>3313951312</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D17" t="n">
         <v>24589067394</v>
       </c>
     </row>
@@ -904,7 +1100,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Petrobras saldo total US$</t>
+          <t>Petrobras saldo US$</t>
         </is>
       </c>
       <c r="B1" t="n">
@@ -914,11 +1110,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Brasil saldo total US$</t>
+          <t>Brasil saldo US$</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62513358693</v>
+        <v>284697957984</v>
       </c>
     </row>
   </sheetData>

</xml_diff>